<commit_message>
Sync planning SharePoint : S18
</commit_message>
<xml_diff>
--- a/Plannings 2026 S18.xlsx
+++ b/Plannings 2026 S18.xlsx
@@ -8642,13 +8642,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BF6C81E-0D71-4705-B02D-03D2D301B281}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A69048A-FE9A-4547-B799-0913FED60783}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B429926D-8763-49D6-AE3A-D7D9A3EFECAC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F706AEFA-B1CD-430D-84D8-22CA09D4DBE5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D071264C-CB3B-418A-BE16-40A8650BF8CD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{813CB447-FC46-4A66-96F2-63C6F9CBC36C}"/>
 </file>
</xml_diff>